<commit_message>
Update OpenF1 lightweight source closure artifacts
</commit_message>
<xml_diff>
--- a/latest/openf1_lightweight_source_closure/F1_OpenF1_Lightweight_Source_Closure_Summary.xlsx
+++ b/latest/openf1_lightweight_source_closure/F1_OpenF1_Lightweight_Source_Closure_Summary.xlsx
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4195</v>
+        <v>4081</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1239</v>
+        <v>1034</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28324</v>
+        <v>58118</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10179</v>
+        <v>6912</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2187</v>
+        <v>1861</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>479</v>
+        <v>509</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H415"/>
+  <dimension ref="A1:H433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4083,7 +4083,7 @@
         <v>1</v>
       </c>
       <c r="G99" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
@@ -4287,11 +4287,11 @@
         <v>1</v>
       </c>
       <c r="G105" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -4389,11 +4389,11 @@
         <v>1</v>
       </c>
       <c r="G108" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -5307,11 +5307,11 @@
         <v>1</v>
       </c>
       <c r="G135" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5375,11 +5375,11 @@
         <v>1</v>
       </c>
       <c r="G137" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5409,11 +5409,11 @@
         <v>1</v>
       </c>
       <c r="G138" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5443,11 +5443,11 @@
         <v>1</v>
       </c>
       <c r="G139" t="n">
-        <v>0</v>
+        <v>20663</v>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5477,11 +5477,11 @@
         <v>1</v>
       </c>
       <c r="G140" t="n">
-        <v>0</v>
+        <v>524</v>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5511,11 +5511,11 @@
         <v>1</v>
       </c>
       <c r="G141" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5545,11 +5545,11 @@
         <v>1</v>
       </c>
       <c r="G142" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
         <v>1</v>
       </c>
       <c r="G144" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H144" t="inlineStr">
         <is>
@@ -5681,11 +5681,11 @@
         <v>1</v>
       </c>
       <c r="G146" t="n">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -5715,11 +5715,11 @@
         <v>1</v>
       </c>
       <c r="G147" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -5783,11 +5783,11 @@
         <v>1</v>
       </c>
       <c r="G149" t="n">
-        <v>709</v>
+        <v>0</v>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -5817,11 +5817,11 @@
         <v>1</v>
       </c>
       <c r="G150" t="n">
-        <v>94</v>
+        <v>0</v>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
         <v>1</v>
       </c>
       <c r="G180" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H180" t="inlineStr">
         <is>
@@ -7449,11 +7449,11 @@
         <v>1</v>
       </c>
       <c r="G198" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -7755,11 +7755,11 @@
         <v>1</v>
       </c>
       <c r="G207" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -8367,11 +8367,11 @@
         <v>1</v>
       </c>
       <c r="G225" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -8673,11 +8673,11 @@
         <v>1</v>
       </c>
       <c r="G234" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -9285,11 +9285,11 @@
         <v>1</v>
       </c>
       <c r="G252" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -9591,11 +9591,11 @@
         <v>1</v>
       </c>
       <c r="G261" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -9897,11 +9897,11 @@
         <v>1</v>
       </c>
       <c r="G270" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -10203,11 +10203,11 @@
         <v>1</v>
       </c>
       <c r="G279" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10271,11 +10271,11 @@
         <v>1</v>
       </c>
       <c r="G281" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10305,11 +10305,11 @@
         <v>1</v>
       </c>
       <c r="G282" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10373,11 +10373,11 @@
         <v>1</v>
       </c>
       <c r="G284" t="n">
-        <v>670</v>
+        <v>0</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10407,11 +10407,11 @@
         <v>1</v>
       </c>
       <c r="G285" t="n">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10509,11 +10509,11 @@
         <v>1</v>
       </c>
       <c r="G288" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10577,11 +10577,11 @@
         <v>1</v>
       </c>
       <c r="G290" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -10611,11 +10611,11 @@
         <v>1</v>
       </c>
       <c r="G291" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11121,11 +11121,11 @@
         <v>1</v>
       </c>
       <c r="G306" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11189,11 +11189,11 @@
         <v>1</v>
       </c>
       <c r="G308" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11223,11 +11223,11 @@
         <v>1</v>
       </c>
       <c r="G309" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11291,11 +11291,11 @@
         <v>1</v>
       </c>
       <c r="G311" t="n">
-        <v>0</v>
+        <v>981</v>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -11733,11 +11733,11 @@
         <v>1</v>
       </c>
       <c r="G324" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11801,11 +11801,11 @@
         <v>1</v>
       </c>
       <c r="G326" t="n">
-        <v>102</v>
+        <v>0</v>
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11835,11 +11835,11 @@
         <v>1</v>
       </c>
       <c r="G327" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11903,11 +11903,11 @@
         <v>1</v>
       </c>
       <c r="G329" t="n">
-        <v>843</v>
+        <v>0</v>
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -11937,11 +11937,11 @@
         <v>1</v>
       </c>
       <c r="G330" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12039,11 +12039,11 @@
         <v>1</v>
       </c>
       <c r="G333" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -12345,11 +12345,11 @@
         <v>1</v>
       </c>
       <c r="G342" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12413,11 +12413,11 @@
         <v>1</v>
       </c>
       <c r="G344" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12447,11 +12447,11 @@
         <v>1</v>
       </c>
       <c r="G345" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12481,11 +12481,11 @@
         <v>1</v>
       </c>
       <c r="G346" t="n">
-        <v>0</v>
+        <v>9131</v>
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12515,11 +12515,11 @@
         <v>1</v>
       </c>
       <c r="G347" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12549,11 +12549,11 @@
         <v>1</v>
       </c>
       <c r="G348" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -12583,11 +12583,11 @@
         <v>1</v>
       </c>
       <c r="G349" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>zero_rows</t>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -13263,11 +13263,11 @@
         <v>1</v>
       </c>
       <c r="G369" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13297,11 +13297,11 @@
         <v>1</v>
       </c>
       <c r="G370" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13331,11 +13331,11 @@
         <v>1</v>
       </c>
       <c r="G371" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13365,11 +13365,11 @@
         <v>1</v>
       </c>
       <c r="G372" t="n">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13433,11 +13433,11 @@
         <v>1</v>
       </c>
       <c r="G374" t="n">
-        <v>1015</v>
+        <v>0</v>
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13467,11 +13467,11 @@
         <v>1</v>
       </c>
       <c r="G375" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -13569,7 +13569,7 @@
         <v>1</v>
       </c>
       <c r="G378" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="H378" t="inlineStr">
         <is>
@@ -14045,11 +14045,11 @@
         <v>1</v>
       </c>
       <c r="G392" t="n">
-        <v>592</v>
+        <v>0</v>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -14079,11 +14079,11 @@
         <v>1</v>
       </c>
       <c r="G393" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -14181,11 +14181,11 @@
         <v>1</v>
       </c>
       <c r="G396" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -14215,11 +14215,11 @@
         <v>1</v>
       </c>
       <c r="G397" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -14249,11 +14249,11 @@
         <v>1</v>
       </c>
       <c r="G398" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -14283,11 +14283,11 @@
         <v>1</v>
       </c>
       <c r="G399" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -14351,11 +14351,11 @@
         <v>1</v>
       </c>
       <c r="G401" t="n">
-        <v>1616</v>
+        <v>0</v>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>zero_rows</t>
         </is>
       </c>
     </row>
@@ -14832,6 +14832,618 @@
       <c r="H415" t="inlineStr">
         <is>
           <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="B416" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C416" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F416" t="b">
+        <v>1</v>
+      </c>
+      <c r="G416" t="n">
+        <v>0</v>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>race_control</t>
+        </is>
+      </c>
+      <c r="B417" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C417" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F417" t="b">
+        <v>1</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0</v>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>intervals</t>
+        </is>
+      </c>
+      <c r="B418" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C418" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F418" t="b">
+        <v>1</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0</v>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="B419" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C419" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F419" t="b">
+        <v>1</v>
+      </c>
+      <c r="G419" t="n">
+        <v>0</v>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>stints</t>
+        </is>
+      </c>
+      <c r="B420" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C420" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F420" t="b">
+        <v>1</v>
+      </c>
+      <c r="G420" t="n">
+        <v>0</v>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>pit</t>
+        </is>
+      </c>
+      <c r="B421" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C421" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F421" t="b">
+        <v>0</v>
+      </c>
+      <c r="G421" t="n">
+        <v>0</v>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>skipped_not_applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>starting_grid</t>
+        </is>
+      </c>
+      <c r="B422" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C422" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F422" t="b">
+        <v>1</v>
+      </c>
+      <c r="G422" t="n">
+        <v>0</v>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>drivers</t>
+        </is>
+      </c>
+      <c r="B423" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C423" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F423" t="b">
+        <v>1</v>
+      </c>
+      <c r="G423" t="n">
+        <v>18</v>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>team_radio</t>
+        </is>
+      </c>
+      <c r="B424" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C424" t="n">
+        <v>11300</v>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F424" t="b">
+        <v>1</v>
+      </c>
+      <c r="G424" t="n">
+        <v>6</v>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="B425" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C425" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F425" t="b">
+        <v>1</v>
+      </c>
+      <c r="G425" t="n">
+        <v>85</v>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>race_control</t>
+        </is>
+      </c>
+      <c r="B426" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C426" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F426" t="b">
+        <v>1</v>
+      </c>
+      <c r="G426" t="n">
+        <v>52</v>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>intervals</t>
+        </is>
+      </c>
+      <c r="B427" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C427" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F427" t="b">
+        <v>1</v>
+      </c>
+      <c r="G427" t="n">
+        <v>0</v>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="B428" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C428" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F428" t="b">
+        <v>1</v>
+      </c>
+      <c r="G428" t="n">
+        <v>424</v>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>stints</t>
+        </is>
+      </c>
+      <c r="B429" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C429" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F429" t="b">
+        <v>1</v>
+      </c>
+      <c r="G429" t="n">
+        <v>118</v>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>pit</t>
+        </is>
+      </c>
+      <c r="B430" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C430" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F430" t="b">
+        <v>0</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0</v>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>skipped_not_applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>starting_grid</t>
+        </is>
+      </c>
+      <c r="B431" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C431" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F431" t="b">
+        <v>1</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0</v>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>zero_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>drivers</t>
+        </is>
+      </c>
+      <c r="B432" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C432" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F432" t="b">
+        <v>1</v>
+      </c>
+      <c r="G432" t="n">
+        <v>22</v>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>team_radio</t>
+        </is>
+      </c>
+      <c r="B433" t="n">
+        <v>1287</v>
+      </c>
+      <c r="C433" t="n">
+        <v>11301</v>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="F433" t="b">
+        <v>1</v>
+      </c>
+      <c r="G433" t="n">
+        <v>6</v>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
     </row>
@@ -14893,11 +15505,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4195</v>
+        <v>4081</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>cc8c69791e6855efc7065a8872a4ab903a1325a7b33d85128f68f1e49b41e28f</t>
+          <t>56ba49a019af8554a4ecc9508eb94c2a70967f97dad7906426d41351d65eefb8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -14923,11 +15535,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1239</v>
+        <v>1034</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6cf53eb51aefd15d9c70465f499a8ba1770bba08b7b7442bddc17e3c5e21ede5</t>
+          <t>22fc80118750717f52c6d0c5136e34ffd06e491e76fde850a74a8c9e49b401fb</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -14953,11 +15565,11 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28324</v>
+        <v>58118</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>343345dc92bc26079449276f72c6ec61d8423a11ff243facc4a624c3cde21b2d</t>
+          <t>5ebe1ac9d2a64b2d46fe20fd93ca442a4aa4ce474deb5ee6ff9fea8e8be4e688</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -14983,11 +15595,11 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10179</v>
+        <v>6912</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5c7908201f48f0742d240a4a9d3c4496d6d82d0616177bb7bc9e3579e2728709</t>
+          <t>8ff2ca8a0da40c13644cd234eec36bfcf9ae2bbacf056edd9226e3dc68fff817</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -15013,11 +15625,11 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2187</v>
+        <v>1861</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>83cbcaddde403d9867ca7ca1f0d9ce8c83afe68239153f1befa4a34b5cdbfa78</t>
+          <t>4688ea9f6e59899460e2f2c6f5cce6f83ac37820c436f19606871283c45bd503</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -15043,11 +15655,11 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>dfcba5f67065e5a2adb89367563b21ca355e83e070fbf98fab7c7a1eab6614ea</t>
+          <t>8b0da5d189330f0124d209989d7520843e46a6e0ae4b7d575d7f2d50a36234a7</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -15103,11 +15715,11 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>479</v>
+        <v>509</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>e01f2ad8379d793e11bc0cb7fb483e3973e1d47ebe95ae05979c21e1af88899e</t>
+          <t>e3801b908a10ab9c68740de83593f544bdace8eca835adc5682a88f7f0fa19c2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -15133,11 +15745,11 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>07548b2dfa24b8b8680138dd329c2b3f7dbb859084b6b8cf5350bd3192358175</t>
+          <t>e89a67b2469fdc6171f5f3a798e288252df3467570cf0bbe9f2885dc2f09d2cc</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -15162,7 +15774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P47"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18375,6 +18987,142 @@
         <v>1</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>11300</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Practice 1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-06-12T11:30:00+00:00</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-06-12T12:30:00+00:00</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G48" t="n">
+        <v>15</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Catalunya</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="O48" t="b">
+        <v>0</v>
+      </c>
+      <c r="P48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>11301</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Practice 2</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-06-12T15:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-06-12T16:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G49" t="n">
+        <v>15</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Catalunya</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>02:00:00</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>2026</v>
+      </c>
+      <c r="O49" t="b">
+        <v>0</v>
+      </c>
+      <c r="P49" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>